<commit_message>
Calculate duck commission after discount
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/internal/kachyni-stravy-chornomorka/demo/chornomorka_duck_dishes_demo.xlsx
+++ b/internal/kachyni-stravy-chornomorka/demo/chornomorka_duck_dishes_demo.xlsx
@@ -511,13 +511,13 @@
         <v>224</v>
       </c>
       <c r="F2" t="n">
-        <v>48</v>
+        <v>33.6</v>
       </c>
       <c r="G2" t="n">
-        <v>32</v>
+        <v>22.4</v>
       </c>
       <c r="H2" t="n">
-        <v>16</v>
+        <v>11.2</v>
       </c>
     </row>
   </sheetData>
@@ -686,13 +686,13 @@
         <v>15</v>
       </c>
       <c r="N2" t="n">
-        <v>48</v>
+        <v>33.6</v>
       </c>
       <c r="O2" t="n">
-        <v>32</v>
+        <v>22.4</v>
       </c>
       <c r="P2" t="n">
-        <v>16</v>
+        <v>11.2</v>
       </c>
     </row>
   </sheetData>
@@ -768,7 +768,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Комісія 15% на качині страви мінус комісія 10% на качині страви</t>
+          <t>5% від вартості доставлених качиних страв після знижки (15% мінус 10%)</t>
         </is>
       </c>
     </row>

</xml_diff>